<commit_message>
CORE-000021: rule verified, updates made to yaml, test data and use of [ABSENT] for record level
</commit_message>
<xml_diff>
--- a/rules/CORE-000021/negative/01/data/unit-test-coreid-CG0397-negative.xlsx
+++ b/rules/CORE-000021/negative/01/data/unit-test-coreid-CG0397-negative.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marisa_wyckmans\CORE\CDISC_Rule_Authoring\core-contributor\rules\CORE-000021\negative\01\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B7789F5-41F7-491B-AECB-249070488BFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1845F24E-7968-4A35-B77E-0BC88798C3C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -501,7 +501,7 @@
     <t>IEDRVFL</t>
   </si>
   <si>
-    <t>Not in dataset</t>
+    <t>[ABSENT]</t>
   </si>
 </sst>
 </file>

</xml_diff>